<commit_message>
Add 8 new job sites to 3D Job Sites tab
Adds PocketGamer.biz Jobs, GameDevMap, CGVerse, CGTrader Jobs, Upwork,
We Work Remotely, Remote Rocketship and Arc.dev (52 sites total).
Updates CSV copy and README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hbx9Uv3bkUWLeb1LDSHAtj
</commit_message>
<xml_diff>
--- a/US_3D_Design_Studios.xlsx
+++ b/US_3D_Design_Studios.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Design Studios'!$A$1:$L$116</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3D Job Sites'!$A$1:$H$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3D Job Sites'!$A$1:$H$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -52,7 +52,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -129,6 +129,11 @@
         <fgColor rgb="00F6F6EA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF7F7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -142,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -281,6 +286,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7865,7 +7882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9144,7 +9161,7 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9184,7 +9201,7 @@
       </c>
       <c r="H33" s="35" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9241,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9264,7 +9281,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9304,7 +9321,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9344,7 +9361,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9384,7 +9401,7 @@
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9424,7 +9441,7 @@
       </c>
       <c r="H39" s="46" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9464,7 +9481,7 @@
       </c>
       <c r="H40" s="46" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9504,7 +9521,7 @@
       </c>
       <c r="H41" s="49" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9540,7 +9557,7 @@
       </c>
       <c r="H42" s="49" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9576,7 +9593,7 @@
       </c>
       <c r="H43" s="49" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9612,7 +9629,7 @@
       </c>
       <c r="H44" s="49" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
         </is>
       </c>
     </row>
@@ -9652,12 +9669,332 @@
       </c>
       <c r="H45" s="49" t="inlineStr">
         <is>
-          <t>From other agent's list</t>
+          <t>From other agent's list (#1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>PocketGamer.biz Jobs</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pocketgamer.jobs</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Mobile and cross-platform game studios</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Run by PocketGamer.biz. Lists 3D environment, prop and technical art roles.</t>
+        </is>
+      </c>
+      <c r="G46" s="52" t="inlineStr">
+        <is>
+          <t>Not checked — site blocks automated reading</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>From other agent's list (#2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="17" t="inlineStr">
+        <is>
+          <t>GameDevMap</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gamedevmap.com</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Finding game studios by location</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Not a job board — a map/directory of game studios. Use it to find studios near Seattle, then check their careers pages. Active (says ~100,000 users in 2025).</t>
+        </is>
+      </c>
+      <c r="G47" s="33" t="inlineStr">
+        <is>
+          <t>Yes — live, saw current jobs</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>From other agent's list (#2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>CGVerse Job Search</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>https://cgverse.com/jobs</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Concept, 3D and technical art roles</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Run by an online art school. Most listings are pulled from ArtStation, so expect overlap with ArtStation Jobs. Saw current roles from Crytek, Ubisoft and Visual Concepts.</t>
+        </is>
+      </c>
+      <c r="G48" s="33" t="inlineStr">
+        <is>
+          <t>Yes — live, saw current jobs</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>From other agent's list (#2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>CGTrader Jobs</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cgtrader.com/3d-modeling-jobs/browse</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Design agencies &amp; product</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Contract 3D modeling tasks</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>3D model marketplace with a job/project board. Page loaded, but listings didn't show.</t>
+        </is>
+      </c>
+      <c r="G49" s="34" t="inlineStr">
+        <is>
+          <t>Site loads, but I couldn't see listings</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>From other agent's list (#2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="53" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="54" t="inlineStr">
+        <is>
+          <t>Upwork</t>
+        </is>
+      </c>
+      <c r="C50" s="55" t="inlineStr">
+        <is>
+          <t>https://www.upwork.com</t>
+        </is>
+      </c>
+      <c r="D50" s="53" t="inlineStr">
+        <is>
+          <t>Freelance &amp; remote</t>
+        </is>
+      </c>
+      <c r="E50" s="53" t="inlineStr">
+        <is>
+          <t>Freelance 3D contracts</t>
+        </is>
+      </c>
+      <c r="F50" s="53" t="inlineStr">
+        <is>
+          <t>Lots of low-budget posts. Search specific terms like "Unreal environment", "product visualization", "WebGL 3D".</t>
+        </is>
+      </c>
+      <c r="G50" s="53" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H50" s="53" t="inlineStr">
+        <is>
+          <t>From other agent's list (#2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="54" t="inlineStr">
+        <is>
+          <t>We Work Remotely</t>
+        </is>
+      </c>
+      <c r="C51" s="55" t="inlineStr">
+        <is>
+          <t>https://weworkremotely.com</t>
+        </is>
+      </c>
+      <c r="D51" s="53" t="inlineStr">
+        <is>
+          <t>Freelance &amp; remote</t>
+        </is>
+      </c>
+      <c r="E51" s="53" t="inlineStr">
+        <is>
+          <t>Remote design and 3D roles</t>
+        </is>
+      </c>
+      <c r="F51" s="53" t="inlineStr">
+        <is>
+          <t>Large remote board (42,000+ jobs posted). Has 3D Modeling and 3D Animation skill filters; saw a remote Senior 3D Designer contract role.</t>
+        </is>
+      </c>
+      <c r="G51" s="33" t="inlineStr">
+        <is>
+          <t>Yes — live, saw current jobs</t>
+        </is>
+      </c>
+      <c r="H51" s="53" t="inlineStr">
+        <is>
+          <t>From other agent's list (#2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="54" t="inlineStr">
+        <is>
+          <t>Remote Rocketship</t>
+        </is>
+      </c>
+      <c r="C52" s="55" t="inlineStr">
+        <is>
+          <t>https://www.remoterocketship.com</t>
+        </is>
+      </c>
+      <c r="D52" s="53" t="inlineStr">
+        <is>
+          <t>Freelance &amp; remote</t>
+        </is>
+      </c>
+      <c r="E52" s="53" t="inlineStr">
+        <is>
+          <t>Remote jobs pulled from company careers pages</t>
+        </is>
+      </c>
+      <c r="F52" s="53" t="inlineStr">
+        <is>
+          <t>Active. Use the Design filter and search "3D". Full search may need a free account.</t>
+        </is>
+      </c>
+      <c r="G52" s="33" t="inlineStr">
+        <is>
+          <t>Yes — live, saw current jobs</t>
+        </is>
+      </c>
+      <c r="H52" s="53" t="inlineStr">
+        <is>
+          <t>From other agent's list (#2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="54" t="inlineStr">
+        <is>
+          <t>Arc.dev</t>
+        </is>
+      </c>
+      <c r="C53" s="55" t="inlineStr">
+        <is>
+          <t>https://arc.dev/remote-jobs/3d-artist</t>
+        </is>
+      </c>
+      <c r="D53" s="53" t="inlineStr">
+        <is>
+          <t>Freelance &amp; remote</t>
+        </is>
+      </c>
+      <c r="E53" s="53" t="inlineStr">
+        <is>
+          <t>Technical / real-time 3D and WebGL roles</t>
+        </is>
+      </c>
+      <c r="F53" s="53" t="inlineStr">
+        <is>
+          <t>Mostly for developers. Its 3D Artist page had 0 jobs when checked.</t>
+        </is>
+      </c>
+      <c r="G53" s="34" t="inlineStr">
+        <is>
+          <t>Site loads, but I couldn't see listings</t>
+        </is>
+      </c>
+      <c r="H53" s="53" t="inlineStr">
+        <is>
+          <t>From other agent's list (#2)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H45"/>
+  <autoFilter ref="A1:H53"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -9702,6 +10039,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>